<commit_message>
create funtion in utils file from mail.py file and use
</commit_message>
<xml_diff>
--- a/flipkart_product_details.xlsx
+++ b/flipkart_product_details.xlsx
@@ -451,26 +451,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Acer Aspire 14 AMD Ryzen 5 3500U - (8 GB/256 GB SSD/Windows 11 Ho...more</t>
+          <t>Acer Aspire 14 Intel Core 7 240H - (16 GB/512 GB SSD/Windows 11 H...more</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36990</v>
+        <v>69990</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>₹37,196</t>
+          <t>₹70,296</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Battery Backup: Up to 10 Hours | Battery Cell: 45.6 Wh Li-ion battery | Bluetooth: Yes | Brand: Acer | Clock Speed: 2.1 GHz | Color: Light Silver | Connectivity Features: Wireless LAN 802.11a/b/g/n/ac+ax wireless LAN Bluetooth Yes | Customer: support | Dimensions: 31.27 x 20.66 x 1.94 cm | Disk Drive: Not Available | Display and Audio Features: Touchscreen No Screen Size 35.56 cm (14 inch) Screen Resolution 1920 x 1080 pixel pixel Screen Type 14 inch display with IPS (In-Plane Switching) technology, Full HD 1920 x 1080, Acer ComfyView LED-backlit TFT LCD Speakers 2 Screen Resolution Type Full HD | Expandable Memory: Upgradable up to 32GB | Finger Print Sensor: No | Graphic Processor: AMD Radeon Vega | HDMI Port: 1x HDMI | In the Box: Sales Package 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Is Fragile: No | Is Tablet: No | Keyboard: 80-/81-/84-key Acer keyboard layout with international language support including indicators of Caps Lock and Co-pilot key | Laptop Bag: No | MS Office Provided: No | Model Name: Aspire 14 | Model Number: AS14-39 | OS Architecture: 64 bit | Operating System: Windows 11 Home | Part Number: UN.37ZSI.007 | Pointer Device: Multi-gesture touchpad, supporting two-finger scroll; pinch, multitasking; application commands | Port and Slot Features: USB Port 2 x USB 3.2 Type C Port, 2 x USB 3.2 Gen 1 Type A, 1 x USB 2.0 port Gen 1 HDMI Port 1x HDMI | Power Supply: 65 W Type C adapter | Processor Brand: AMD | Processor Name: Ryzen 5 | Processor Variant: 3500U | Processor and Memory Features: Processor Brand AMD Processor Name Ryzen 5 SSD Yes SSD Capacity 256 GB RAM 8 GB RAM Type DDR4 Processor Variant 3500U Clock Speed 2.1 GHz Expandable Memory Upgradable up to 32GB Graphic Processor AMD Radeon Vega Storage Type SSD Operating System Windows 11 Home | RAM: 8 GB | RAM Type: DDR4 | SSD: Yes | SSD Capacity: 256 GB | Sales Package: 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Screen Resolution: 1920 x 1080 pixel pixel | Screen Resolution Type: Full HD | Screen Size: 35.56 cm (14 inch) | Screen Type: 14 inch display with IPS (In-Plane Switching) technology, Full HD 1920 x 1080, Acer ComfyView LED-backlit TFT LCD | Series: Aspire 14 | Speakers: 2 | Storage Type: SSD | Suitable For: Performance, Processing &amp; Multitasking, Everyday Use, Travel &amp; Business | System Architecture: 64 | Touchscreen: No | Type: Notebook | USB Port: 2 x USB 3.2 Type C Port, 2 x USB 3.2 Gen 1 Type A, 1 x USB 2.0 port Gen 1 | Web Camera: HD camera | Weight: 1.45 kg | Wireless LAN: 802.11a/b/g/n/ac+ax wireless LAN</t>
+          <t>Battery Cell: 54Wh Li-ion battery | Bluetooth: Yes | Brand: Acer | Clock Speed: 2.5 GHz | Color: Pure Silver | Connectivity Features: Wireless LAN 802.11a/b/g/n/ac+ax wireless LAN Bluetooth Yes | Dimensions: 31.4.4 x 21.98 x 2.03 cm | Disk Drive: Not Available | Display and Audio Features: Touchscreen No Screen Size 35.56 cm (14 inch) Screen Resolution 1920 x 1200 pixel pixel Screen Type 14 inch display with IPS (In-Plane Switching) technology, WUXGA 1920 x 1200, Acer ComfyView LED-backlit TFT LCD Speakers 2 Screen Resolution Type WUXGA | Finger Print Sensor: No | Graphic Processor: Intel Graphics | HDMI Port: 1x HDMI | In the Box: Sales Package 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Included Software: MSO | Is Fragile: No | Is Tablet: No | Keyboard: 80-/81-/84-key Acer backlit keyboard layout with international language support including indicators of CapsLock and Co-pilot key | Laptop Bag: No | MS Office Provided: Yes | Model Name: Aspire 14 | Model Number: AS14H-53 | OS Architecture: 64 bit | Operating System: Windows 11 Home | Part Number: UN.36CSI.00B | Pointer Device: Multi-gesture touchpad, supporting two-finger scroll; pinch; gestures to open Cortana, Action Center, multitasking; application commands | Port and Slot Features: USB Port 1 x USB 3.2 port Type C, 3 x USB 3.0 port Gen 1, 2 x USB 3.0 HDMI Port 1x HDMI | Power Supply: 90 W AC adapter | Processor Brand: Intel | Processor Name: Core 7 | Processor Variant: 240H | Processor and Memory Features: Processor Brand Intel Processor Name Core 7 SSD Yes SSD Capacity 512 GB RAM 16 GB RAM Type LPDDR5 Processor Variant 240H Clock Speed 2.5 GHz Graphic Processor Intel Graphics Storage Type SSD Operating System Windows 11 Home | RAM: 16 GB | RAM Type: LPDDR5 | SSD: Yes | SSD Capacity: 512 GB | Sales Package: 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Screen Resolution: 1920 x 1200 pixel pixel | Screen Resolution Type: WUXGA | Screen Size: 35.56 cm (14 inch) | Screen Type: 14 inch display with IPS (In-Plane Switching) technology, WUXGA 1920 x 1200, Acer ComfyView LED-backlit TFT LCD | Series: Aspire 14 | Speakers: 2 | Storage Type: SSD | Suitable For: Performance, Processing &amp; Multitasking, Everyday Use, Travel &amp; Business | System Architecture: 64 | Touchscreen: No | Type: Notebook | USB Port: 1 x USB 3.2 port Type C, 3 x USB 3.0 port Gen 1, 2 x USB 3.0 | Web Camera: HD camera | Weight: 1.44 kg | Wireless LAN: 802.11a/b/g/n/ac+ax wireless LAN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hardening and edge-case resilience for all product categories
</commit_message>
<xml_diff>
--- a/flipkart_product_details.xlsx
+++ b/flipkart_product_details.xlsx
@@ -451,26 +451,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Acer Aspire 14 Intel Core 7 240H - (16 GB/512 GB SSD/Windows 11 H...more</t>
+          <t>Samsung Galaxy Book4 Metal Intel Core i5 13th Gen 1335U - (16 GB/512 GB SSD/Windows 11 Home) NP750XGJ</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69990</v>
+        <v>60990</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>₹70,296</t>
+          <t>₹61,296</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Battery Cell: 54Wh Li-ion battery | Bluetooth: Yes | Brand: Acer | Clock Speed: 2.5 GHz | Color: Pure Silver | Connectivity Features: Wireless LAN 802.11a/b/g/n/ac+ax wireless LAN Bluetooth Yes | Dimensions: 31.4.4 x 21.98 x 2.03 cm | Disk Drive: Not Available | Display and Audio Features: Touchscreen No Screen Size 35.56 cm (14 inch) Screen Resolution 1920 x 1200 pixel pixel Screen Type 14 inch display with IPS (In-Plane Switching) technology, WUXGA 1920 x 1200, Acer ComfyView LED-backlit TFT LCD Speakers 2 Screen Resolution Type WUXGA | Finger Print Sensor: No | Graphic Processor: Intel Graphics | HDMI Port: 1x HDMI | In the Box: Sales Package 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Included Software: MSO | Is Fragile: No | Is Tablet: No | Keyboard: 80-/81-/84-key Acer backlit keyboard layout with international language support including indicators of CapsLock and Co-pilot key | Laptop Bag: No | MS Office Provided: Yes | Model Name: Aspire 14 | Model Number: AS14H-53 | OS Architecture: 64 bit | Operating System: Windows 11 Home | Part Number: UN.36CSI.00B | Pointer Device: Multi-gesture touchpad, supporting two-finger scroll; pinch; gestures to open Cortana, Action Center, multitasking; application commands | Port and Slot Features: USB Port 1 x USB 3.2 port Type C, 3 x USB 3.0 port Gen 1, 2 x USB 3.0 HDMI Port 1x HDMI | Power Supply: 90 W AC adapter | Processor Brand: Intel | Processor Name: Core 7 | Processor Variant: 240H | Processor and Memory Features: Processor Brand Intel Processor Name Core 7 SSD Yes SSD Capacity 512 GB RAM 16 GB RAM Type LPDDR5 Processor Variant 240H Clock Speed 2.5 GHz Graphic Processor Intel Graphics Storage Type SSD Operating System Windows 11 Home | RAM: 16 GB | RAM Type: LPDDR5 | SSD: Yes | SSD Capacity: 512 GB | Sales Package: 1 x Laptop, 1 x Power Adaptor, 1 x User Guide, 1 x Warranty Documents | Screen Resolution: 1920 x 1200 pixel pixel | Screen Resolution Type: WUXGA | Screen Size: 35.56 cm (14 inch) | Screen Type: 14 inch display with IPS (In-Plane Switching) technology, WUXGA 1920 x 1200, Acer ComfyView LED-backlit TFT LCD | Series: Aspire 14 | Speakers: 2 | Storage Type: SSD | Suitable For: Performance, Processing &amp; Multitasking, Everyday Use, Travel &amp; Business | System Architecture: 64 | Touchscreen: No | Type: Notebook | USB Port: 1 x USB 3.2 port Type C, 3 x USB 3.0 port Gen 1, 2 x USB 3.0 | Web Camera: HD camera | Weight: 1.44 kg | Wireless LAN: 802.11a/b/g/n/ac+ax wireless LAN</t>
+          <t>Additional Features: Disk Drive Not Available Web Camera Yes, 1 Megapixel Finger Print Sensor Yes Keyboard QWERTY | Battery Cell: 4 Cell Lithium Ion Battery | Bluetooth: v5.2 | Brand: Samsung | Clock Speed: Max Frequency Up to 4.60 GHz | Color: Gray | Connectivity Features: Wireless LAN 802.11ax Bluetooth v5.2 | Dimensions: 356.6 x 15.4 x 229.15mm | Disk Drive: Not Available | Display and Audio Features: Touchscreen No Screen Size 39.62 cm (15.6 Inch) Screen Resolution 1920 x 1080 Pixel Screen Type Full HD LCD Display Speakers HD Audio Codec, Dolby Atmos, Embedded Stereo Speakers, Internal Digital MIC Internal Mic Internal Digital MIC Refresh Rate 60 Hz Screen Resolution Type Full HD | Finger Print Sensor: Yes | Graphic Processor: Intel Integrated Iris Xe | HDMI Port: Yes, 1 x HDMI | In the Box: Sales Package Laptop, 45W Charger, Data Cable(USB-C to C, 1.8m), Quick Start Guide | Intel Core i5 13th Gen: Experience lightning-fast speed | Intel Integrated: Efficient graphics for everyday use | Internal Mic: Internal Digital MIC | Is Fragile: No | Is Tablet: No | Keyboard: QWERTY | MS Office Provided: Yes | Mic In: Yes | Model Name: NP750XGJ-LG7IN | Model Number: NP750XGJ | OS Architecture: 64 bit | Operating System: Windows 11 Home | Part Number: NP750XGJ-KG2IN / NP750XGJ-LG2IN /NP750XGJ-LS6IN | Port and Slot Features: Mic In Yes USB Port Yes, 2 x USB Type C, 2 x USB 3.2 Type A HDMI Port Yes, 1 x HDMI | Power Supply: 45W AC Adapter | Processor Brand: Intel | Processor Generation: 13th Gen | Processor Name: Core i5 | Processor Variant: 1335U | Processor and Memory Features: Processor Brand Intel Processor Name Core i5 Processor Generation 13th Gen SSD Yes SSD Capacity 512 GB RAM 16 GB RAM Type LPDDR4X Processor Variant 1335U Clock Speed Max Frequency Up to 4.60 GHz Graphic Processor Intel Integrated Iris Xe Storage Type SSD Operating System Windows 11 | RAM: 16 GB | RAM Type: LPDDR4X | Refresh Rate: 60 Hz | SSD: Yes | SSD Capacity: 512 GB | Sales Package: Laptop, 45W Charger, Data Cable(USB-C to C, 1.8m), Quick Start Guide | Screen Resolution: 1920 x 1080 Pixel | Screen Resolution Type: Full HD | Screen Size: 39.62 cm (15.6 Inch) | Screen Type: Full HD LCD Display | Series: Galaxy Book4 Metal | Speakers: HD Audio Codec, Dolby Atmos, Embedded Stereo Speakers, Internal Digital MIC | Storage Type: SSD | Suitable For: Processing &amp; Multitasking | Touchscreen: No | Type: Thin and Light Laptop | USB Port: Yes, 2 x USB Type C, 2 x USB 3.2 Type A | Web Camera: Yes, 1 Megapixel | Weight: 1.55 Kg | Wireless LAN: 802.11ax</t>
         </is>
       </c>
     </row>

</xml_diff>